<commit_message>
Fix UART alignment bug on GCS causing multiple phantom reads per second
</commit_message>
<xml_diff>
--- a/AI_AuditLog_Template.xlsx
+++ b/AI_AuditLog_Template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12375" activeTab="3"/>
+    <workbookView windowWidth="19200" windowHeight="8150"/>
   </bookViews>
   <sheets>
     <sheet name="1. Metadata &amp; Summary" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="214">
   <si>
     <t>AI AUDIT LOG - METADATA &amp; SUMMARY</t>
   </si>
@@ -28,15 +28,13 @@
     <t>Student Name:</t>
   </si>
   <si>
-    <t>Nguyễn Ngọc Duy
-Huỳnh Quốc Cường</t>
+    <t>Kiều Chấn Đông</t>
   </si>
   <si>
     <t>Student ID:</t>
   </si>
   <si>
-    <t>SE205008
-SE205311</t>
+    <t>SE201124</t>
   </si>
   <si>
     <t>Course:</t>
@@ -48,7 +46,7 @@
     <t>Assignment:</t>
   </si>
   <si>
-    <t>Weather Station Monitoring System</t>
+    <t>Environmental Monitoring Drone Based</t>
   </si>
   <si>
     <t>AI USAGE SUMMARY</t>
@@ -57,18 +55,12 @@
     <t>Total Prompts Used (all AI tools):</t>
   </si>
   <si>
-    <t>~90</t>
-  </si>
-  <si>
     <t>Core Prompts Logged:</t>
   </si>
   <si>
     <t>Selection Ratio:</t>
   </si>
   <si>
-    <t>Should be 10-20%</t>
-  </si>
-  <si>
     <t>Hallucination Detected:</t>
   </si>
   <si>
@@ -108,7 +100,22 @@
     <t>Speed up coding</t>
   </si>
   <si>
-    <t>[Add more...]</t>
+    <t>Google Gemini</t>
+  </si>
+  <si>
+    <t>Hardware debugging, architectual advise</t>
+  </si>
+  <si>
+    <t>Deep technical analysist of hardware-software interaction</t>
+  </si>
+  <si>
+    <t>Anthropic Claude</t>
+  </si>
+  <si>
+    <t>Code review, logic optimization</t>
+  </si>
+  <si>
+    <t>High-quality code generation and logic refinement</t>
   </si>
   <si>
     <t>CORE PROMPTS DISTRIBUTION BY DTC COMPONENT</t>
@@ -171,146 +178,268 @@
     <t>001</t>
   </si>
   <si>
-    <t xml:space="preserve">QUYẾT ĐỊNH
-</t>
-  </si>
-  <si>
-    <t>Lựa chọn phần cứng (Hardware Selection)</t>
-  </si>
-  <si>
-    <t>Nhóm cần chọn vi điều khiển chính: Arduino Uno hay ESP32 để điều khiển toàn bộ hệ thống.</t>
-  </si>
-  <si>
-    <t>Arduino Uno hay ESP32 phù hợp hơn cho dự án khóa cửa thông minh có cảm biến vân tay, bàn phím, Bluetooth và servo?</t>
-  </si>
-  <si>
-    <t>AI đề xuất dùng ESP32 vì: có WiFi và Bluetooth tích hợp sẵn, nhiều bộ nhớ hơn, xử lý nhanh hơn, phù hợp với các dự án IoT hiện đại.</t>
-  </si>
-  <si>
-    <t>Tư duy phản biện: ESP32 mạnh hơn thật, nhưng dự án đã có module HC-05 xử lý Bluetooth rồi, nên WiFi/BT tích hợp của ESP32 không cần thiết.
- Bối cảnh hóa: Nhóm quen dùng Arduino Uno, chuyển sang ESP32 sẽ mất thêm thời gian học. Thời gian dự án chỉ có 11 tuần.
- Sáng tạo tổng hợp: So sánh cụ thể — Arduino Uno: 16MHz, 2KB RAM, giá ~70k; ESP32: 240MHz, 520KB RAM, giá ~90k. Với 6 thiết bị ngoại vi của nhóm, Arduino Uno hoàn toàn đủ dùng.
- Quyết định: Giữ Arduino Uno. Gợi ý của AI đúng với dự án lớn hơn, nhưng với quy mô dự án này, Uno là lựa chọn hợp lý và tiết kiệm thời gian hơn.</t>
-  </si>
-  <si>
-    <t>Bảng so sánh thông số Arduino Uno và ESP32; danh sách 6 thiết bị ngoại vi của nhóm</t>
+    <t xml:space="preserve">DECISION
+</t>
+  </si>
+  <si>
+    <t>Algorithm Design (Data Processing)</t>
+  </si>
+  <si>
+    <t>The BMP280 pressure was displayed in hPa, but we wanted Pascal (Pa). The forecast algorithm also needed to be scaled accordingly.</t>
+  </si>
+  <si>
+    <t>Please ensure everywhere in the project, including the serial monitor, pressure is in Pa to match the BMP280, and check the altitude calculation.</t>
+  </si>
+  <si>
+    <t>AI provided a multi-file replacement plan, removing the `/ 100.0F` division, updating HTML UI to "Pa", and scaling the JS forecast thresholds (e.g., 1013 to 101300).</t>
+  </si>
+  <si>
+    <t>Critical Thinking: The AI correctly identified all files needing changes. Contextualization: Scaling the JS thresholds was crucial to prevent the forecast logic from breaking. Synthesis &amp; Decision: Applied the changes, ensuring consistency across C++, HTML, and JS.</t>
+  </si>
+  <si>
+    <t>Github commit reverting pressure to raw Pascal (Pa).</t>
   </si>
   <si>
     <t>002</t>
   </si>
   <si>
-    <t>QUYẾT ĐỊNH</t>
-  </si>
-  <si>
-    <t>Lựa chọn giao thức (Bluetooth vs WiFi MQTT)</t>
-  </si>
-  <si>
-    <t>Nhóm cần chọn cách điện thoại giao tiếp với khóa cửa: dùng Bluetooth HC-05 hay WiFi kết hợp MQTT.</t>
-  </si>
-  <si>
-    <t>Nên dùng Bluetooth HC-05 hay WiFi MQTT để điều khiển khóa cửa từ điện thoại?</t>
-  </si>
-  <si>
-    <t>AI đề xuất dùng WiFi MQTT vì: điều khiển được từ xa bất kỳ đâu trên thế giới, lưu lịch sử lên cloud, là chuẩn phổ biến trong IoT.</t>
-  </si>
-  <si>
-    <t>Tư duy phản biện: WiFi MQTT cần có internet ổn định. Nếu mạng bị mất, khóa cửa không điều khiển được — đây là rủi ro an toàn nghiêm trọng.
- Bối cảnh hóa: Khóa cửa đặt ngay cửa nhà. Người dùng luôn đứng trong vòng 10 mét khi dùng, nên phạm vi Bluetooth là quá đủ.
- Sáng tạo tổng hợp: Bluetooth HC-05 phản hồi dưới 50ms, không cần internet. WiFi MQTT mất 150–400ms và phụ thuộc vào đường truyền mạng. Với khóa cửa, độ tin cậy quan trọng hơn khả năng điều khiển từ xa.
- Quyết định: Giữ Bluetooth HC-05. AI gợi ý tốt cho hệ thống smart home phức tạp, nhưng không phù hợp với khóa cửa đơn giản cần hoạt động offline.</t>
-  </si>
-  <si>
-    <t>Datasheet HC-05; bảng so sánh độ trễ Bluetooth vs MQTT</t>
-  </si>
-  <si>
-    <t>GIẢI QUYẾT VẤN ĐỀ</t>
-  </si>
-  <si>
-    <t>Lỗi đăng ký vân tay (Fingerprint Enrollment Bug)</t>
-  </si>
-  <si>
-    <t>Khi đăng ký vân tay mới, bước quét lần 2 luôn thất bại, dẫn đến không lưu được mẫu vân tay.</t>
-  </si>
-  <si>
-    <t>Tại sao hàm enrollFingerprint() luôn thất bại ở lần quét thứ 2? Đây là code của nhóm: [dán code vào]</t>
-  </si>
-  <si>
-    <t>AI tìm ra lỗi: biến 'p' không được đặt lại về -1 trước vòng lặp quét lần 2. Do đó vòng lặp nghĩ là đã quét xong và bỏ qua hoàn toàn. Ngoài ra, code không nhắc người dùng nhấc ngón tay ra giữa 2 lần quét.</t>
-  </si>
-  <si>
-    <t>Tư duy phản biện: AI chẩn đoán đúng. Kiểm tra lại code thấy đoạn xử lý lần 2 bị comment out từ lúc debug và quên bật lại.
- Bối cảnh hóa: Cảm biến AS608 cần 2 lần quét từ 2 góc hơi khác nhau để tạo mẫu vân tay tốt. Bỏ qua bước này khiến mẫu kém chất lượng, dẫn đến từ chối vân tay đúng nhiều lần.
- Sáng tạo tổng hợp: Khôi phục đoạn code bị comment, thêm lệnh 'p = -1' trước vòng lặp thứ 2, thêm delay 2 giây với thông báo LCD 'Nhấc ngón tay...'. Thử nghiệm với 5 ngón tay khác nhau.
- Quyết định: Áp dụng sửa lỗi. Tỷ lệ đăng ký thành công tăng từ ~40% lên 100%. Đây là trường hợp AI giúp nhóm phát hiện lỗi mà nhóm bỏ sót trong quá trình review code.</t>
-  </si>
-  <si>
-    <t>Code trước và sau khi sửa; kết quả thử nghiệm: 40% → 100% tỷ lệ đăng ký thành công</t>
-  </si>
-  <si>
-    <t>Xung đột cổng UART – Bluetooth và USB Debug</t>
-  </si>
-  <si>
-    <t>Lệnh gửi qua Bluetooth bị nhiễu và sai dữ liệu khi cắm cáp USB vào Arduino để debug.</t>
-  </si>
-  <si>
-    <t>HC-05 đang dùng chân D0/D1 (hardware Serial), đồng thời cũng dùng Serial để debug qua USB. Lệnh Bluetooth bị lỗi khi cắm USB. Cách sửa?</t>
-  </si>
-  <si>
-    <t>AI gợi ý: chuyển HC-05 sang SoftwareSerial trên chân D2 và D3 để giải phóng hardware Serial cho USB. Ví dụ: SoftwareSerial BTSerial(2, 3);</t>
-  </si>
-  <si>
-    <t>Tư duy phản biện: Ý tưởng của AI đúng về nguyên tắc, nhưng chân D2 và D3 đã được cảm biến vân tay dùng rồi (SoftwareSerial fingerSerial(2, 3) trong code hiện tại). Làm theo AI sẽ tạo ra xung đột mới.
- Bối cảnh hóa: Arduino Uno chỉ có 1 cổng hardware Serial. Nhóm có 2 thiết bị dùng serial (vân tay + Bluetooth) nên phải lên kế hoạch phân chân rất cẩn thận.
- Sáng tạo tổng hợp: Lập bảng phân chân đầy đủ — D4–D11 dùng cho bàn phím, A4–A5 dùng cho LCD I2C, D2–D3 dùng cho vân tay. Chân còn trống an toàn: D13 và A3. Chuyển HC-05 sang SoftwareSerial(13, A3).
- Quyết định: Chuyển HC-05 sang chân D13/A3. AI đưa ra hướng đúng nhưng không kiểm tra code sẵn có của nhóm trước khi gợi ý. Nhóm phải tự phân tích toàn bộ bảng phân chân.</t>
-  </si>
-  <si>
-    <t>Bảng phân chân đầy đủ của hệ thống; sơ đồ mạch đã cập nhật</t>
-  </si>
-  <si>
-    <t>KIỂM CHỨNG</t>
-  </si>
-  <si>
-    <t>Lỗ hổng bảo mật – Phím A reset mật khẩu không cần xác thực</t>
-  </si>
-  <si>
-    <t>Phát hiện ra rằng nhấn phím 'A' trên bàn phím sẽ reset mật khẩu về '1234' mà không cần nhập mật khẩu hiện tại.</t>
-  </si>
-  <si>
-    <t>Đây có phải lỗ hổng bảo mật không? Phím A reset mật khẩu về 1234 mà không kiểm tra gì cả. Đây là code: [dán vào]</t>
-  </si>
-  <si>
-    <t>AI xác nhận: đây là lỗ hổng bảo mật nghiêm trọng. Bất kỳ ai chạm được vào bàn phím đều có thể reset mật khẩu và mở khóa cửa. Cách sửa: yêu cầu nhập mật khẩu admin trước, giống như các phím B, C, D.</t>
-  </si>
-  <si>
-    <t>Tư duy phản biện: Nhóm thử nghiệm thực tế — nhấn phím A khi hệ thống đang chạy, mật khẩu reset ngay lập tức. Lỗ hổng hoàn toàn có thể khai thác được.
- Bối cảnh hóa: Đây có lẽ là phím tắt được thêm vào để tiện reset trong lúc test, và bị quên không xóa đi trước khi ra sản phẩm cuối.
- Sáng tạo tổng hợp: Sửa đơn giản — chuyển logic phím A vào trong khối kiểm tra mật khẩu admin. Nhóm cũng phát hiện thêm vấn đề: khi mất điện, bộ đếm số lần nhập sai bị xóa, cho phép bypass cơ chế khóa bằng cách ngắt nguồn.
- Quyết định: Đã sửa phím A. Vấn đề bypass khi mất điện được ghi nhận là hạn chế đã biết. Hướng cải thiện tương lai: lưu số lần nhập sai vào EEPROM.</t>
-  </si>
-  <si>
-    <t>Code trước và sau khi sửa; log thử nghiệm xác nhận lỗ hổng và bản vá</t>
-  </si>
-  <si>
-    <t>AI bịa tài liệu tham khảo (Hallucination – Fake Citation)</t>
-  </si>
-  <si>
-    <t>Nhóm nhờ AI gợi ý bài báo IEEE về xác thực đa lớp (vân tay + PIN) trên thiết bị IoT để đưa vào phần tài liệu tham khảo của báo cáo.</t>
-  </si>
-  <si>
-    <t>Tìm cho tôi một bài báo IEEE về xác thực đa lớp kết hợp vân tay và mã PIN trên hệ thống nhúng hoặc IoT.</t>
-  </si>
-  <si>
-    <t>AI gợi ý: 'Zhang et al. (2023), Multi-factor Authentication for Smart Home IoT Devices, IEEE Transactions on Consumer Electronics.' Kèm theo tóm tắt nội dung và các số liệu hiệu năng cụ thể.</t>
-  </si>
-  <si>
-    <t>Tư duy phản biện: PHÁT HIỆN ẢO GIÁC AI. Nhóm tìm trên IEEE Xplore với đúng tiêu đề và tên tác giả — không có kết quả nào. Bài báo không tồn tại. AI đã bịa hoàn toàn.
- Bối cảnh hóa: Đây là lỗi phổ biến của AI với tài liệu học thuật — tạo ra tên bài báo, tên tác giả và tên tạp chí nghe rất thật nhưng không có thật. Nếu dùng trong báo cáo sẽ là vi phạm học thuật nghiêm trọng.
- Sáng tạo tổng hợp: Nhóm tự tìm trên IEEE Xplore với từ khóa 'fingerprint authentication IoT embedded'. Tìm được 2 bài báo thật: Abuhamad et al. (2021) trên IEEE Access và Mohsin et al. (2020) trên IEEE IoT Journal.
- Quyết định: Thay thế tài liệu giả bằng 2 bài báo đã xác minh. Quy tắc mới của nhóm: không bao giờ trích dẫn tài liệu mà chưa tự tìm và mở ra đọc trực tiếp trên cơ sở dữ liệu học thuật.</t>
-  </si>
-  <si>
-    <t>Ảnh chụp màn hình tìm kiếm IEEE Xplore (không có kết quả cho Zhang 2023); link PDF 2 bài báo thật</t>
+    <t>PROBLEM-SOLVING</t>
+  </si>
+  <si>
+    <t>Pattern Recognition (Cloud Integration)</t>
+  </si>
+  <si>
+    <t>The GCS ESP32 was failing to upload to ThingSpeak, throwing HTTP error -301 despite having the correct API key.</t>
+  </si>
+  <si>
+    <t>I entered the correct ID and API key, but my account hasn't been added to the channel. Is this the cause of error -301?</t>
+  </si>
+  <si>
+    <t>AI confirmed that ThingSpeak uses an ownership model, so if the account is not added as a contributor to the channel, it will reject the Write API Key with a -301 error.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI correctly pinpointed the -301 error code as an authentication failure, not a network issue. Contextualization: The project uses a shared team channel, requiring contributor access. Decision: Asked the channel owner to grant write access to my email, solving the issue.</t>
+  </si>
+  <si>
+    <t>ThingSpeak channel sharing settings &amp; successful upload logs.</t>
+  </si>
+  <si>
+    <t>003</t>
+  </si>
+  <si>
+    <t>Decomposition (Hardware Debugging)</t>
+  </si>
+  <si>
+    <t>HC-12 radio communication failed. Payload was sending AT but getting no OK. GCS was receiving garbage characters (square boxes).</t>
+  </si>
+  <si>
+    <t>On the left is payload, right is GCS. Payload sends little, GCS receives garbage. Payload doesn't receive what GCS sends.</t>
+  </si>
+  <si>
+    <t>AI identified a baud rate mismatch. It broke the problem down, explaining that garbage chars mean RF is working but baud is mismatched. It provided step-by-step instructions to factory reset both HC-12s using the SET pin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Critical Thinking: AI's deduction that garbage = successful RF link but wrong baud rate was spot on. Decomposition: We separated the GCS and Payload troubleshooting, resetting them one by one. Decision: Followed the reset procedure to sync both modules to 9600 baud.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serial monitor screenshots showing garbage chars vs clean text.
+</t>
+  </si>
+  <si>
+    <t>004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Algorithm Design (Serial Communication)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sending AT to HC-12 via the Serial Monitor yielded no OK response during the reset procedure.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At the payload, I send AT but receive nothing.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI recognized that println() was appending \r\n, which choked the HC-12 AT parser. It provided a pure byte-for-byte passthrough algorithm (write(read())) to bypass string formatting.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Critical Thinking: The standard readStringUntil logic was modifying the raw commands. Algorithm Design: The pure passthrough loop is a much more robust algorithm for configuring hardware modules. Decision: Rewrote the test scripts to pure passthrough, and successfully entered AT mode.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commit "Rewrite HC12 tests to pure UART passthrough".
+</t>
+  </si>
+  <si>
+    <t>005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decomposition (Power Management)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Payload ESP32 continuously rebooted whenever the ENV Mode (Environment Mode) was turned on.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When uploading payload code, everything is normal until I turn ENV mode on, then the payload auto-resets continuously.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI decomposed the ENV_MODE_ON trigger and identified the DHT11 sensor as the culprit. Hypothesized a hardware short circuit pulling the 3.3V rail low when ESP32 drives the DHT11 data pin, causing a brownout reset. Suggested unplugging DHT11 to isolate the fault.
+</t>
+  </si>
+  <si>
+    <t>Critical Thinking: The AI didn't blame the code but recognized a hardware brownout pattern. Decomposition: Isolating the DHT11 by unplugging it immediately stopped the reboots, confirming the hypothesis. Decision: Re-wired the DHT11 correctly.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serial logs showing boot loops stopping after DHT11 removal.
+</t>
+  </si>
+  <si>
+    <t>006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pattern Recognition (Sensor Interfacing)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">After fixing the reset issue, the BMP280 and DHT11 both returned nan (Not a Number), while the SRF05 altitude worked fine.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Except for altitude, all other parameters are nan, whereas yesterday it worked.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI recognized the pattern: both nan sensors run on 3.3V. It deduced that while unplugging the DHT11, I likely accidentally unplugged the shared 3.3V or GND wire on the breadboard, killing power to the BMP280 as well.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Critical Thinking: AI correctly mapped the nan software error to a physical power rail disconnection. Pattern Recognition: Both failed sensors shared the same power rail, while the working one (SRF05) used 5V. Decision: Pushed the jumper wires firmly into the 3.3V rail, restoring sensor data.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screenshot of nan values and subsequent valid readings.
+</t>
+  </si>
+  <si>
+    <t>007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROBLEM-SOLVING
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pattern Recognition (UART Noise)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The HC-12 on the payload started printing a continuous, infinite stream of square boxes without any user input.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HC-12 on payload is failing again (infinite square boxes on screen).
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI identified the classic pattern of a "floating RX pin" or a disconnected GND wire between the HC-12 and ESP32, which acts as an antenna picking up electromagnetic noise and interpreting it as random UART bytes.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Critical Thinking: Infinite garbage without input is a distinct hardware noise signature. Pattern Recognition: AI matched this to a floating ground or RX pin. Decision: Reconnected the loose GND wire on the HC-12, immediately stopping the garbage spam.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serial monitor screenshot showing infinite square boxes.
+</t>
+  </si>
+  <si>
+    <t>008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Algorithm Design (UART Framing)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The atomizer was flashing on and off unstably when turned on, despite GCS sending valid commands.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I notice the atomizer flashes on and off instead of staying on continuously. Please check the code flow.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI analyzed the UART buffer and found a logic flaw: clearing the backlog blindly caused packet misalignment. It designed a frame synchronization algorithm using peek() == 1 to align incoming data with the GCSCommand struct.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Critical Thinking: The AI found a subtle race condition in UART parsing where partial packets corrupted the struct fields. Algorithm Design: Implementing a sync byte is a standard and robust algorithm for serial protocols. Decision: Applied the frame sync fix, completely resolving the flickering.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commit "Fix UART alignment bug causing atomizer to flicker".
+</t>
+  </si>
+  <si>
+    <t>009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abstraction (System Architecture)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evaluating the power distribution layout: BMP280, HC-12, DHT11 on 3.3V; SRF05 and Atomizer on VIN (5V).
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Currently BMP280, HC-12, DHT11 are on 3.3v and SRF05, Atomizer on VIN. Do you see anything wrong?
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI praised the layout, explaining the abstraction of "Power Isolation". Putting the HC-12 on the 3.3V LDO regulator filters out the massive voltage spikes caused by the 5V Atomizer, ensuring radio stability. Also noted that 3.3V sensors perfectly match the ESP32's logic level.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Critical Thinking: AI highlighted the hidden benefits of power isolation and logic level matching. Abstraction: Viewing the 3.3V LDO as a noise filter rather than just a power source was a great architectural insight. Decision: Kept the power distribution exactly as is.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hardware schematic and stable operation logs.
+</t>
+  </si>
+  <si>
+    <t>010</t>
+  </si>
+  <si>
+    <t>VERIFICATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abstraction (Safety Mechanisms)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wanted to add a fail-safe notification on the Payload if it loses connection with the GCS.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I want to add a notification line on the payload if it doesn't receive a signal from GCS, so I know to fix it.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI abstracted the connection state by implementing a software watchdog. It tracked last_rx_time and added logic to print a warning every 3 seconds if the timeout is exceeded.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Critical Thinking: A simple timeout check is highly effective and non-blocking. Abstraction: Abstracting connection lost to a simple millis() delta avoids complex bidirectional ping-pong protocols. Decision: Added the watchdog code, which successfully alerted me when I turned off the GCS.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commit "Add connection timeout warning to Payload serial monitor".
+</t>
   </si>
   <si>
     <t>HALLUCINATION DETECTION LOG (BẮT BUỘC)</t>
@@ -337,34 +466,115 @@
     <t>Corrective Action</t>
   </si>
   <si>
-    <t>Hiểu sai bối cảnh (Context Misunderstanding)</t>
-  </si>
-  <si>
-    <t>AI gợi ý chuyển HC-05 sang SoftwareSerial trên chân D2 và D3 để sửa xung đột UART.</t>
-  </si>
-  <si>
-    <t>Chân D2 và D3 đã được cảm biến vân tay sử dụng trong code hiện tại. Làm theo AI sẽ tạo ra xung đột mới.</t>
-  </si>
-  <si>
-    <t>Nhóm kiểm tra lại toàn bộ code và phát hiện dòng 'SoftwareSerial fingerSerial(2, 3)' đã chiếm D2/D3 từ trước. AI không đọc code sẵn có trước khi đề xuất.</t>
-  </si>
-  <si>
-    <t>Lập bảng phân chân đầy đủ cho tất cả 7 thiết bị ngoại vi. Tìm ra chân D13 và A3 là 2 chân còn trống an toàn. Chuyển HC-05 sang SoftwareSerial(13, A3).</t>
-  </si>
-  <si>
-    <t>Bịa tài liệu tham khảo (Fabrication – Fake Citation)</t>
-  </si>
-  <si>
-    <t>AI nói rằng bài báo 'Zhang et al. (2023), Multi-factor Authentication for Smart Home IoT Devices, IEEE Transactions on Consumer Electronics' tồn tại và có các số liệu hiệu năng cụ thể.</t>
-  </si>
-  <si>
-    <t>Bài báo này không tồn tại. Tìm kiếm trên IEEE Xplore với đúng tiêu đề và tên tác giả không ra kết quả nào.</t>
-  </si>
-  <si>
-    <t>Nhóm tự tìm trên IEEE Xplore, Google Scholar và ResearchGate với tiêu đề đầy đủ và rút gọn — đều không có kết quả. Đây là dạng ảo giác phổ biến nhất của AI với tài liệu học thuật.</t>
-  </si>
-  <si>
-    <t>Tìm thủ công trên IEEE Xplore và xác minh được 2 bài báo thật liên quan. Đặt quy tắc nhóm: mọi tài liệu tham khảo phải được tự tìm và mở ra đọc trên cơ sở dữ liệu học thuật trước khi trích dẫn.</t>
+    <t xml:space="preserve">Fabrication (Fake Citation)
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI suggested reading a paper titled "UAV-based Environmental Monitoring Frameworks" by Nguyen et al. 2023, IEEE Sensors.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The paper does not exist. A search on IEEE Xplore yielded no results for that title or author combination.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Searched the exact title on Google Scholar and IEEE Xplore.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ignored the fake citation and manually searched IEEE for real papers on drone environmental monitoring.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Context Misunderstanding
+</t>
+  </si>
+  <si>
+    <t>AI suggested using WiFi.begin() on the Payload ESP32 to transmit sensor data directly to the cloud.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The drone payload operates high in the air, far outside the range of any home WiFi network. It MUST use the HC-12 radio to send data to the GCS on the ground.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviewed the project architecture diagram which clearly shows Payload -&gt; HC-12 -&gt; GCS -&gt; WiFi.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rejected the WiFi code and prompted the AI to use HC12Serial.write() instead.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hardware Capability Hallucination
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI stated the ESP32 can supply up to 2 Amps from its 3.3V pin to power the Atomizer directly.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The ESP32 onboard AMS1117 3.3V regulator maxes out at ~600mA-800mA. Drawing 2A would instantly fry the regulator.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Checked the ESP32 DevKit V1 schematic and the AMS1117 datasheet.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Powered the Atomizer directly from a dedicated 5V buck converter and controlled it via a MOSFET.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Software API Hallucination
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI provided code using HC12Serial.setBaudRate(9600) to dynamically change the radio baud rate on the fly.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The HC-12 module does not support software-only baud rate changes via an API method. It requires the physical SET pin to be pulled LOW to enter AT command mode.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Checked the SoftwareSerial/HardwareSerial documentation and the HC-12 datasheet.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ignored the fake method and manually wired the SET pin to GND to send AT+DEFAULT.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI suggested adding delay(2000) in the main loop to wait for the DHT11 sensor to stabilize between readings.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Using a 2-second blocking delay in the same loop that forwards flight commands to the Flight Controller would cause the drone to crash instantly due to control unresponsiveness.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traced the FreeRTOS task execution flow and realized delay() blocks the entire task.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaced the blocking delay with a non-blocking millis() timer or vTaskDelay on a separate FreeRTOS task.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI suggested connecting the HC-12 TX pin to GPIO 34 on the ESP32 for UART communication.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIOs 34, 35, 36, 39 on the ESP32 are INPUT-ONLY pins. They lack the internal circuitry to output data, so TX cannot function on GPIO 34.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consulted the ESP32 pinout diagram which marks pins 34-39 as input only.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Re-assigned the HC-12 TX/RX pins to GPIO 32 and 33, which support full bidirectional UART.
+</t>
   </si>
   <si>
     <t>HALLUCINATION TYPES REFERENCE:</t>
@@ -424,7 +634,7 @@
     <t>Không biết business constraints</t>
   </si>
   <si>
-    <t>awd</t>
+    <t>SELF-ASSESSMENT CHECKLIST</t>
   </si>
   <si>
     <t>Kiểm tra kỹ trước khi nộp. MỖI ENTRY phải pass ≥4/5 tiêu chí dưới đây.</t>
@@ -451,7 +661,7 @@
     <t>Prompt này ảnh hưởng đến quyết định quan trọng trong project?</t>
   </si>
   <si>
-    <t>☐</t>
+    <t>x</t>
   </si>
   <si>
     <t>2</t>
@@ -521,9 +731,6 @@
   </si>
   <si>
     <t>Tôi có evidence?</t>
-  </si>
-  <si>
-    <t>003</t>
   </si>
 </sst>
 </file>
@@ -532,10 +739,10 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
     <numFmt numFmtId="176" formatCode="0.0%"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="36">
     <font>
@@ -667,16 +874,25 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
+      <color theme="3"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -684,29 +900,6 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -721,7 +914,53 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -735,55 +974,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -798,14 +997,22 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF006100"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -850,7 +1057,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8"/>
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -862,7 +1081,97 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -874,7 +1183,43 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -886,145 +1231,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1085,32 +1292,6 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top/>
       <bottom style="medium">
         <color theme="4"/>
@@ -1135,9 +1316,44 @@
     <border>
       <left/>
       <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top/>
       <bottom style="medium">
         <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1156,25 +1372,16 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1186,134 +1393,134 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="17" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="27" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="30" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="30" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="29" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="29" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1355,11 +1562,14 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1370,10 +1580,16 @@
     <xf numFmtId="0" fontId="15" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="176" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1638,15 +1854,15 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F999"/>
-  <sheetFormatPr defaultColWidth="14.4285714285714" defaultRowHeight="15" customHeight="1" outlineLevelCol="5"/>
+  <dimension ref="A1:F1001"/>
+  <sheetFormatPr defaultColWidth="14.4272727272727" defaultRowHeight="15" customHeight="1" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
     <col min="5" max="6" width="20" customWidth="1"/>
-    <col min="7" max="26" width="8.71428571428571" customWidth="1"/>
+    <col min="7" max="26" width="8.71818181818182" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="21" spans="1:1">
@@ -1654,13 +1870,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" ht="18.75" spans="1:1">
+    <row r="3" ht="18.5" spans="1:1">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" ht="29.25" customHeight="1" spans="1:3">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="24" t="s">
         <v>2</v>
       </c>
       <c r="C4" t="s">
@@ -1668,15 +1884,15 @@
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="24" t="s">
         <v>4</v>
       </c>
       <c r="C5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="22" t="s">
+    <row r="6" ht="14.5" spans="1:3">
+      <c r="A6" s="24" t="s">
         <v>6</v>
       </c>
       <c r="C6" t="s">
@@ -1684,172 +1900,194 @@
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="24" t="s">
         <v>8</v>
       </c>
       <c r="C7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" ht="18.75" spans="1:1">
+    <row r="9" ht="18.5" spans="1:1">
       <c r="A9" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:3">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="24" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="22" t="s">
+      <c r="C11" s="25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="23">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="22" t="s">
+      <c r="C12" s="26">
+        <f>C11/C10</f>
+        <v>0.125</v>
+      </c>
+      <c r="E12" s="27"/>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="24" t="e">
-        <f>C11/C10</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E12" s="25" t="s">
+      <c r="C13" s="25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" ht="18.5" spans="1:1">
+      <c r="A15" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
-      <c r="A13" s="22" t="s">
+    <row r="16" ht="14.5" spans="1:4">
+      <c r="A16" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" ht="18.75" spans="1:1">
-      <c r="A15" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="4" t="s">
+      <c r="C16" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="4" t="s">
+    </row>
+    <row r="17" ht="29" spans="1:4">
+      <c r="A17" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D16" s="4" t="s">
+      <c r="B17" s="14" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="17" ht="30" spans="1:4">
-      <c r="A17" s="14" t="s">
+      <c r="C17" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="D17" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="14" t="s">
+    </row>
+    <row r="18" ht="14.5" spans="1:4">
+      <c r="A18" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="B18" s="14" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="14" t="s">
+      <c r="C18" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="D18" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C18" s="14" t="s">
+    </row>
+    <row r="19" ht="29" spans="1:4">
+      <c r="A19" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="B19" s="14" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="14" t="s">
+      <c r="C19" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D19" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-    </row>
-    <row r="20" ht="15.75" customHeight="1"/>
-    <row r="21" ht="15.75" customHeight="1" spans="1:1">
-      <c r="A21" s="3" t="s">
+    </row>
+    <row r="20" ht="29" spans="1:4">
+      <c r="A20" s="28" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1" spans="1:3">
-      <c r="A22" s="4" t="s">
+      <c r="B20" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="C20" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="D20" s="28" t="s">
         <v>32</v>
       </c>
-      <c r="C22" s="4" t="s">
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="28"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="28"/>
+    </row>
+    <row r="22" ht="15.75" customHeight="1"/>
+    <row r="23" ht="15.75" customHeight="1" spans="1:1">
+      <c r="A23" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="23" ht="15.75" customHeight="1" spans="1:3">
-      <c r="A23" s="14" t="s">
+    <row r="24" ht="15.75" customHeight="1" spans="1:3">
+      <c r="A24" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B23" s="26">
-        <v>2</v>
-      </c>
-      <c r="C23" s="13" t="s">
+      <c r="B24" s="4" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" spans="1:3">
-      <c r="A24" s="14" t="s">
+      <c r="C24" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="B24" s="26">
-        <v>3</v>
-      </c>
-      <c r="C24" s="13" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" spans="1:3">
       <c r="A25" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="B25" s="26">
+      <c r="B25" s="29">
         <v>2</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" spans="1:3">
       <c r="A26" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B26" s="29">
+        <v>3</v>
+      </c>
+      <c r="C26" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="26">
+    </row>
+    <row r="27" ht="15.75" customHeight="1" spans="1:3">
+      <c r="A27" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="29">
+        <v>2</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1" spans="1:3">
+      <c r="A28" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" s="29">
         <v>3</v>
       </c>
-      <c r="C26" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1"/>
-    <row r="28" ht="15.75" customHeight="1"/>
+      <c r="C28" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
     <row r="29" ht="15.75" customHeight="1"/>
     <row r="30" ht="15.75" customHeight="1"/>
     <row r="31" ht="15.75" customHeight="1"/>
@@ -2821,6 +3059,8 @@
     <row r="997" ht="15.75" customHeight="1"/>
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
+    <row r="1000" ht="15.75" customHeight="1"/>
+    <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
@@ -2835,249 +3075,313 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:H1000"/>
-  <sheetFormatPr defaultColWidth="14.4285714285714" defaultRowHeight="15" customHeight="1" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="14.4272727272727" defaultRowHeight="15" customHeight="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="35" customWidth="1"/>
-    <col min="7" max="7" width="65.4285714285714" customWidth="1"/>
+    <col min="7" max="7" width="65.4272727272727" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
-    <col min="9" max="26" width="8.71428571428571" customWidth="1"/>
+    <col min="9" max="26" width="8.71818181818182" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="21" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:1">
-      <c r="A2" s="19" t="s">
-        <v>40</v>
+      <c r="A2" s="20" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="3" ht="39.75" customHeight="1" spans="1:8">
       <c r="A3" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" ht="99.75" customHeight="1" spans="1:8">
       <c r="A4" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>50</v>
+        <v>52</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>53</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H4" s="18" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" ht="99.75" customHeight="1" spans="1:8">
       <c r="A5" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="B5" s="21" t="s">
-        <v>58</v>
+        <v>60</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>61</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E5" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="G5" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="H5" s="18" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" ht="99.75" customHeight="1" spans="1:8">
+      <c r="A6" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="F5" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="G5" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="H5" s="18" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="6" ht="99.75" customHeight="1" spans="1:8">
-      <c r="A6" s="14">
-        <v>3</v>
-      </c>
-      <c r="B6" s="21" t="s">
-        <v>65</v>
-      </c>
       <c r="C6" s="18" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="H6" s="18" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" ht="79.5" customHeight="1" spans="1:8">
-      <c r="A7" s="14">
-        <v>4</v>
-      </c>
-      <c r="B7" s="21" t="s">
-        <v>65</v>
+      <c r="A7" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>61</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="H7" s="18" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" ht="79.5" customHeight="1" spans="1:8">
-      <c r="A8" s="14">
-        <v>5</v>
-      </c>
-      <c r="B8" s="21" t="s">
-        <v>78</v>
+      <c r="A8" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>61</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="H8" s="18" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" ht="79.5" customHeight="1" spans="1:8">
-      <c r="A9" s="14">
-        <v>6</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>78</v>
+      <c r="A9" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>61</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="H9" s="18" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10" ht="79.5" customHeight="1" spans="1:8">
-      <c r="A10" s="14"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
+      <c r="A10" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="G10" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H10" s="14" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="11" ht="79.5" customHeight="1" spans="1:8">
-      <c r="A11" s="14"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
+      <c r="A11" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="B11" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="G11" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="H11" s="14" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="12" ht="79.5" customHeight="1" spans="1:8">
-      <c r="A12" s="14"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
+      <c r="A12" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="B12" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="F12" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="G12" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="H12" s="14" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="13" ht="79.5" customHeight="1" spans="1:8">
-      <c r="A13" s="14"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
+      <c r="A13" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="B13" s="23" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="F13" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="G13" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="H13" s="14" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="14" ht="79.5" customHeight="1" spans="1:8">
       <c r="A14" s="14"/>
@@ -4198,115 +4502,163 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F1000"/>
-  <sheetFormatPr defaultColWidth="14.4285714285714" defaultRowHeight="15" customHeight="1" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="14.4272727272727" defaultRowHeight="15" customHeight="1" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="6" width="30" customWidth="1"/>
-    <col min="7" max="26" width="8.71428571428571" customWidth="1"/>
+    <col min="7" max="26" width="8.71818181818182" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="21" spans="1:1">
       <c r="A1" s="15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" ht="14.5" spans="1:1">
       <c r="A2" s="16" t="s">
-        <v>92</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" ht="39.75" customHeight="1" spans="1:6">
       <c r="A3" s="4" t="s">
-        <v>93</v>
+        <v>128</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>94</v>
+        <v>129</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>95</v>
+        <v>130</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>96</v>
+        <v>131</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>97</v>
+        <v>132</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>98</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1" spans="1:6">
-      <c r="A4" s="17">
-        <v>4</v>
+      <c r="A4" s="17" t="s">
+        <v>52</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>99</v>
+        <v>134</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>100</v>
+        <v>135</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>101</v>
+        <v>136</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>102</v>
+        <v>137</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="5" ht="90" spans="1:6">
-      <c r="A5" s="17">
-        <v>6</v>
+        <v>138</v>
+      </c>
+    </row>
+    <row r="5" ht="87" spans="1:6">
+      <c r="A5" s="17" t="s">
+        <v>60</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>104</v>
+        <v>139</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>105</v>
+        <v>140</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>106</v>
+        <v>141</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>107</v>
+        <v>142</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>108</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" ht="60" customHeight="1" spans="1:6">
-      <c r="A6" s="14"/>
-      <c r="B6" s="14"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
+      <c r="A6" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="7" ht="60" customHeight="1" spans="1:6">
-      <c r="A7" s="14"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
+      <c r="A7" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>153</v>
+      </c>
     </row>
     <row r="8" ht="60" customHeight="1" spans="1:6">
-      <c r="A8" s="14"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
+      <c r="A8" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="9" ht="60" customHeight="1" spans="1:6">
-      <c r="A9" s="14"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
+      <c r="A9" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="10" ht="60" customHeight="1" spans="1:6">
       <c r="A10" s="14"/>
@@ -4435,73 +4787,73 @@
     <row r="29" ht="15.75" customHeight="1"/>
     <row r="30" ht="15.75" customHeight="1" spans="1:1">
       <c r="A30" s="3" t="s">
-        <v>109</v>
+        <v>162</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" spans="1:3">
       <c r="A31" s="12" t="s">
-        <v>110</v>
+        <v>163</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>111</v>
+        <v>164</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>112</v>
+        <v>165</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" spans="1:3">
       <c r="A32" s="14" t="s">
-        <v>113</v>
+        <v>166</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>114</v>
+        <v>167</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>115</v>
+        <v>168</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1" spans="1:3">
       <c r="A33" s="14" t="s">
-        <v>116</v>
+        <v>169</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>117</v>
+        <v>170</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>118</v>
+        <v>171</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1" spans="1:3">
       <c r="A34" s="14" t="s">
-        <v>119</v>
+        <v>172</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>120</v>
+        <v>173</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>121</v>
+        <v>174</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1" spans="1:3">
       <c r="A35" s="14" t="s">
-        <v>122</v>
+        <v>175</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>123</v>
+        <v>176</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>124</v>
+        <v>177</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1" spans="1:3">
       <c r="A36" s="14" t="s">
-        <v>125</v>
+        <v>178</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>126</v>
+        <v>179</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>127</v>
+        <v>180</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1"/>
@@ -5483,227 +5835,227 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:D1000"/>
-  <sheetFormatPr defaultColWidth="14.4285714285714" defaultRowHeight="15" customHeight="1" outlineLevelCol="3"/>
+  <sheetFormatPr defaultColWidth="14.4272727272727" defaultRowHeight="15" customHeight="1" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
-    <col min="5" max="26" width="8.71428571428571" customWidth="1"/>
+    <col min="5" max="26" width="8.71818181818182" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="21" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="2" ht="14.5" spans="1:1">
       <c r="A2" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="4" ht="18.75" spans="1:1">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="4" ht="18.5" spans="1:1">
       <c r="A4" s="3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="5" ht="14.5" spans="1:4">
       <c r="A5" s="4" t="s">
-        <v>131</v>
+        <v>184</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>132</v>
+        <v>185</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>133</v>
+        <v>186</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>134</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="6" t="s">
-        <v>135</v>
+        <v>188</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>136</v>
+        <v>189</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>137</v>
+        <v>190</v>
       </c>
       <c r="D6" s="7"/>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="6" t="s">
-        <v>138</v>
+        <v>191</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>139</v>
+        <v>192</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>137</v>
+        <v>190</v>
       </c>
       <c r="D7" s="7"/>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="6" t="s">
-        <v>140</v>
+        <v>193</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>141</v>
+        <v>194</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>137</v>
+        <v>190</v>
       </c>
       <c r="D8" s="7"/>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="6" t="s">
-        <v>142</v>
+        <v>195</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>143</v>
+        <v>196</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>137</v>
+        <v>190</v>
       </c>
       <c r="D9" s="7"/>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="6" t="s">
-        <v>144</v>
+        <v>197</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>145</v>
+        <v>198</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>137</v>
+        <v>190</v>
       </c>
       <c r="D10" s="7"/>
     </row>
-    <row r="12" ht="18.75" spans="1:1">
+    <row r="12" ht="18.5" spans="1:1">
       <c r="A12" s="3" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="13" ht="14.5" spans="1:4">
       <c r="A13" s="4" t="s">
-        <v>131</v>
+        <v>184</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>132</v>
+        <v>185</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>133</v>
+        <v>186</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>147</v>
+        <v>200</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="6" t="s">
-        <v>135</v>
+        <v>188</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>148</v>
+        <v>201</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>137</v>
+        <v>190</v>
       </c>
       <c r="D14" s="7"/>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="6" t="s">
-        <v>138</v>
+        <v>191</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>149</v>
+        <v>202</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>137</v>
+        <v>190</v>
       </c>
       <c r="D15" s="7"/>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="6" t="s">
-        <v>140</v>
+        <v>193</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>150</v>
+        <v>203</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>137</v>
+        <v>190</v>
       </c>
       <c r="D16" s="7"/>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="6" t="s">
-        <v>142</v>
+        <v>195</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>151</v>
+        <v>204</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>137</v>
+        <v>190</v>
       </c>
       <c r="D17" s="7"/>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="6" t="s">
-        <v>144</v>
+        <v>197</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>152</v>
+        <v>205</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>137</v>
+        <v>190</v>
       </c>
       <c r="D18" s="7"/>
     </row>
-    <row r="20" ht="15.75" spans="1:1">
+    <row r="20" ht="15.5" spans="1:1">
       <c r="A20" s="8" t="s">
-        <v>153</v>
+        <v>206</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" spans="1:1">
       <c r="A21" s="9" t="s">
-        <v>154</v>
+        <v>207</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" spans="1:1">
       <c r="A22" s="9" t="s">
-        <v>155</v>
+        <v>208</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1"/>
     <row r="24" ht="15.75" customHeight="1"/>
     <row r="25" ht="15.75" customHeight="1" spans="1:1">
       <c r="A25" s="3" t="s">
-        <v>156</v>
+        <v>209</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" spans="1:1">
       <c r="A26" s="10" t="s">
-        <v>157</v>
+        <v>210</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" spans="1:4">
       <c r="A27" s="11" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>158</v>
+        <v>211</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>159</v>
+        <v>212</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>160</v>
+        <v>213</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" spans="1:4">
       <c r="A28" s="13" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B28" s="14"/>
       <c r="C28" s="14"/>
@@ -5711,7 +6063,7 @@
     </row>
     <row r="29" ht="15.75" customHeight="1" spans="1:4">
       <c r="A29" s="13" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B29" s="14"/>
       <c r="C29" s="14"/>
@@ -5719,7 +6071,7 @@
     </row>
     <row r="30" ht="15.75" customHeight="1" spans="1:4">
       <c r="A30" s="13" t="s">
-        <v>161</v>
+        <v>68</v>
       </c>
       <c r="B30" s="14"/>
       <c r="C30" s="14"/>

</xml_diff>